<commit_message>
Backup database and excel log
</commit_message>
<xml_diff>
--- a/datalog.xlsx
+++ b/datalog.xlsx
@@ -578,7 +578,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC6"/>
+  <dimension ref="A1:AD8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -668,6 +668,9 @@
       <c r="AC1" t="str">
         <v>Sit_Vid fritidsaktivitet</v>
       </c>
+      <c r="AD1" t="str">
+        <v>Liksidig_HNS</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -757,6 +760,9 @@
       <c r="AC2" t="str">
         <v>Aldrig</v>
       </c>
+      <c r="AD2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -846,6 +852,9 @@
       <c r="AC3" t="str">
         <v>Aldrig</v>
       </c>
+      <c r="AD3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -935,6 +944,9 @@
       <c r="AC4" t="str">
         <v>Ibland</v>
       </c>
+      <c r="AD4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -1024,6 +1036,9 @@
       <c r="AC5" t="str">
         <v>Aldrig</v>
       </c>
+      <c r="AD5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1113,10 +1128,197 @@
       <c r="AC6" t="str">
         <v>Sällan</v>
       </c>
+      <c r="AD6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>77</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-05-15</v>
+      </c>
+      <c r="C7" t="str">
+        <v>7-18</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2013</v>
+      </c>
+      <c r="E7" t="str">
+        <v>5.00</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>5.00</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Grav (71-80 dB)</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Grav (71-80 dB)</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Ledningshinder</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Ledningshinder</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Ja</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Ja</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="P7" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="R7" t="str">
+        <v>Bakom örat</v>
+      </c>
+      <c r="S7" t="str">
+        <v>Baha</v>
+      </c>
+      <c r="T7" t="str">
+        <v>Sällan</v>
+      </c>
+      <c r="U7" t="str">
+        <v>Ibland</v>
+      </c>
+      <c r="V7" t="str">
+        <v>Alltid</v>
+      </c>
+      <c r="W7" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="X7" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="Y7" t="str">
+        <v>Sällan</v>
+      </c>
+      <c r="Z7" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="AA7" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="AB7" t="str">
+        <v>Sällan</v>
+      </c>
+      <c r="AC7" t="str">
+        <v>Sällan</v>
+      </c>
+      <c r="AD7" t="str">
+        <v>Ja</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>hello</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-05-03</v>
+      </c>
+      <c r="C8" t="str">
+        <v>7-18</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2012</v>
+      </c>
+      <c r="E8" t="str">
+        <v>99.00</v>
+      </c>
+      <c r="F8" t="str">
+        <v>77.00</v>
+      </c>
+      <c r="G8" t="str">
+        <v>77.00</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Måttlig (41-60 dB)</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Måttlig (41-60 dB)</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Sensorineural</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Sensorineural</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Ja</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Ja</v>
+      </c>
+      <c r="P8" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="R8" t="str">
+        <v>Bakom örat</v>
+      </c>
+      <c r="S8" t="str">
+        <v>Bakom örat</v>
+      </c>
+      <c r="T8" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="U8" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="V8" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="W8" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="X8" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="Y8" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="Z8" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="AA8" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="AB8" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="AC8" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="AD8" t="str">
+        <v>Ja</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clear all session and patient data, reset Excel log
</commit_message>
<xml_diff>
--- a/datalog.xlsx
+++ b/datalog.xlsx
@@ -578,7 +578,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD8"/>
+  <dimension ref="A1:AC6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -668,9 +668,6 @@
       <c r="AC1" t="str">
         <v>Sit_Vid fritidsaktivitet</v>
       </c>
-      <c r="AD1" t="str">
-        <v>Liksidig_HNS</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -760,9 +757,6 @@
       <c r="AC2" t="str">
         <v>Aldrig</v>
       </c>
-      <c r="AD2" t="str">
-        <v/>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -852,9 +846,6 @@
       <c r="AC3" t="str">
         <v>Aldrig</v>
       </c>
-      <c r="AD3" t="str">
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -944,9 +935,6 @@
       <c r="AC4" t="str">
         <v>Ibland</v>
       </c>
-      <c r="AD4" t="str">
-        <v/>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -1036,9 +1024,6 @@
       <c r="AC5" t="str">
         <v>Aldrig</v>
       </c>
-      <c r="AD5" t="str">
-        <v/>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1128,197 +1113,10 @@
       <c r="AC6" t="str">
         <v>Sällan</v>
       </c>
-      <c r="AD6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>77</v>
-      </c>
-      <c r="B7" t="str">
-        <v>2026-05-15</v>
-      </c>
-      <c r="C7" t="str">
-        <v>7-18</v>
-      </c>
-      <c r="D7" t="str">
-        <v>2013</v>
-      </c>
-      <c r="E7" t="str">
-        <v>5.00</v>
-      </c>
-      <c r="F7" t="str">
-        <v/>
-      </c>
-      <c r="G7" t="str">
-        <v>5.00</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Grav (71-80 dB)</v>
-      </c>
-      <c r="I7" t="str">
-        <v>Grav (71-80 dB)</v>
-      </c>
-      <c r="J7" t="str">
-        <v>Ledningshinder</v>
-      </c>
-      <c r="K7" t="str">
-        <v>Ledningshinder</v>
-      </c>
-      <c r="L7" t="str">
-        <v>Ja</v>
-      </c>
-      <c r="M7" t="str">
-        <v>Ja</v>
-      </c>
-      <c r="N7" t="str">
-        <v>Nej</v>
-      </c>
-      <c r="O7" t="str">
-        <v>Nej</v>
-      </c>
-      <c r="P7" t="str">
-        <v>Nej</v>
-      </c>
-      <c r="Q7" t="str">
-        <v>Nej</v>
-      </c>
-      <c r="R7" t="str">
-        <v>Bakom örat</v>
-      </c>
-      <c r="S7" t="str">
-        <v>Baha</v>
-      </c>
-      <c r="T7" t="str">
-        <v>Sällan</v>
-      </c>
-      <c r="U7" t="str">
-        <v>Ibland</v>
-      </c>
-      <c r="V7" t="str">
-        <v>Alltid</v>
-      </c>
-      <c r="W7" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="X7" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="Y7" t="str">
-        <v>Sällan</v>
-      </c>
-      <c r="Z7" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="AA7" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="AB7" t="str">
-        <v>Sällan</v>
-      </c>
-      <c r="AC7" t="str">
-        <v>Sällan</v>
-      </c>
-      <c r="AD7" t="str">
-        <v>Ja</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>hello</v>
-      </c>
-      <c r="B8" t="str">
-        <v>2026-05-03</v>
-      </c>
-      <c r="C8" t="str">
-        <v>7-18</v>
-      </c>
-      <c r="D8" t="str">
-        <v>2012</v>
-      </c>
-      <c r="E8" t="str">
-        <v>99.00</v>
-      </c>
-      <c r="F8" t="str">
-        <v>77.00</v>
-      </c>
-      <c r="G8" t="str">
-        <v>77.00</v>
-      </c>
-      <c r="H8" t="str">
-        <v>Måttlig (41-60 dB)</v>
-      </c>
-      <c r="I8" t="str">
-        <v>Måttlig (41-60 dB)</v>
-      </c>
-      <c r="J8" t="str">
-        <v>Sensorineural</v>
-      </c>
-      <c r="K8" t="str">
-        <v>Sensorineural</v>
-      </c>
-      <c r="L8" t="str">
-        <v>Nej</v>
-      </c>
-      <c r="M8" t="str">
-        <v>Nej</v>
-      </c>
-      <c r="N8" t="str">
-        <v>Ja</v>
-      </c>
-      <c r="O8" t="str">
-        <v>Ja</v>
-      </c>
-      <c r="P8" t="str">
-        <v>Nej</v>
-      </c>
-      <c r="Q8" t="str">
-        <v>Nej</v>
-      </c>
-      <c r="R8" t="str">
-        <v>Bakom örat</v>
-      </c>
-      <c r="S8" t="str">
-        <v>Bakom örat</v>
-      </c>
-      <c r="T8" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="U8" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="V8" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="W8" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="X8" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="Y8" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="Z8" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="AA8" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="AB8" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="AC8" t="str">
-        <v>Aldrig</v>
-      </c>
-      <c r="AD8" t="str">
-        <v>Ja</v>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement patient info and situation assessment form steps with dynamic validation
</commit_message>
<xml_diff>
--- a/datalog.xlsx
+++ b/datalog.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC2"/>
+  <dimension ref="A1:AD2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -435,64 +435,158 @@
         <v>HNS_Type_R</v>
       </c>
       <c r="L1" t="str">
+        <v>Liksidig_HNS</v>
+      </c>
+      <c r="M1" t="str">
         <v>Basnedsattning_L</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Basnedsattning_R</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Diskantnedsattning_L</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Diskantnedsattning_R</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>FlatLoss_L</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>FlatLoss_R</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>HA_Type_L</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>HA_Type_R</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>Sit_Vid måltid</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>Sit_Egen lek</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>Sit_Lek/aktivitet med föräldrar/kompisar</v>
       </c>
-      <c r="W1" t="str">
+      <c r="X1" t="str">
         <v>Sit_TV/dator/surfplatta</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Y1" t="str">
         <v>Sit_Vid läggdags</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="Z1" t="str">
         <v>Sit_I barnvagnen</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AA1" t="str">
         <v>Sit_I bilen</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AB1" t="str">
         <v>Sit_På förskolan</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AC1" t="str">
         <v>Sit_Utomhus</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AD1" t="str">
         <v>Sit_På offentliga platser</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-05-19</v>
+      </c>
+      <c r="C2" t="str">
+        <v>0-6</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2024</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>0.08</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Normal (&lt;20)</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Lätt (26-40 dB)</v>
+      </c>
+      <c r="J2" t="str">
+        <v>---</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Ledningshinder</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Ja</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Nej</v>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v>Baha</v>
+      </c>
+      <c r="U2" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="V2" t="str">
+        <v>Ibland</v>
+      </c>
+      <c r="W2" t="str">
+        <v>Ibland</v>
+      </c>
+      <c r="X2" t="str">
+        <v>Ibland</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="Z2" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="AA2" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="AB2" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="AC2" t="str">
+        <v>Aldrig</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>Aldrig</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>